<commit_message>
Fixed Copilot DOM issue
</commit_message>
<xml_diff>
--- a/validation-api/audit_logs/prompt_audit_log.xlsx
+++ b/validation-api/audit_logs/prompt_audit_log.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1384,6 +1384,180 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25 16:17:54 UTC</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt.com</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Hey, can you help me write an email to our client John Smith at john.smith@acme.com? His phone is 555-123-4567. This is confidential internal project data for Project Phoenix.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>certain parts need correction</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Personal Information; Sensitive Information</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Inclusion of personal contact information (email address and phone number).; Mention of handling confidential internal project data.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25 16:19:11 UTC</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt.com</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Hey, can you help me write an email to our client John Smith at john.smith@acme.com? His phone is 555-123-4567. This is confidential internal project data for Project Phoenix.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>certain parts need correction</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Sensitive Information; Confidential Project Data</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Confidential client contact details were provided without context or authorization.; Inclusion of potentially sensitive project information without anonymization.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25 20:03:16 UTC</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>chatgpt.com</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Hello</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25 20:11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>copilot.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Hello</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25 20:11:58 UTC</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>copilot.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>SIN:12345678</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>certain parts need correction</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Sensitive Personal Information</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>The Social Insurance Number (SIN) is included in the prompt, which violates the policy against allowing SIN.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>